<commit_message>
Add Harvey-Benchmark to week ending 17-Jul-26 (AI investment-decisioning tuck-in)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBdTT3suK4uAL7A2zUGPUX
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -579,7 +579,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Asset &amp; Wealth Tech</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -594,17 +594,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>15-Jul-26</t>
+          <t>16-Jul-26</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>bloXroute Labs</t>
+          <t>Benchmark</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>FalconX</t>
+          <t>Harvey</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Blockchain distribution network delivering low-latency transaction propagation, real-time chain data, and trading connectivity for institutional on-chain trading</t>
+          <t>AI-powered investment-decisioning platform (due-diligence, data-room, and deal-document analysis) for asset managers; tuck-in building out legal-AI firm Harvey's asset-management business</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -682,17 +682,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-26</t>
+          <t>15-Jul-26</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>c. myers corporation</t>
+          <t>bloXroute Labs</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Strata Decision Technology (Roper)</t>
+          <t>FalconX</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
+          <t>Blockchain distribution network delivering low-latency transaction propagation, real-time chain data, and trading connectivity for institutional on-chain trading</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -770,17 +770,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>16-Jul-26</t>
+          <t>14-Jul-26</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Veridas</t>
+          <t>c. myers corporation</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fourthline</t>
+          <t>Strata Decision Technology (Roper)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
+          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -843,92 +843,181 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>16-Jul-26</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Veridas</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Fourthline</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>17-Jul-26</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Strategic M&amp;A</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>14-Jul-26</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Qolo</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>CSI (Computer Services, Inc.)</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>API-based treasury and payments infrastructure unifying card issuing, multi-rail money movement, and real-time ledgering for commercial banks and embedded finance</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R5"/>
+  <autoFilter ref="A1:R6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add AngelList-Ark and RealPage-Cherre from PitchBook Daily Pitch cross-check
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBdTT3suK4uAL7A2zUGPUX
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Asset &amp; Wealth Tech</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -682,17 +682,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>15-Jul-26</t>
+          <t>16-Jul-26</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>bloXroute Labs</t>
+          <t>Ark PES</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>FalconX</t>
+          <t>AngelList</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Blockchain distribution network delivering low-latency transaction propagation, real-time chain data, and trading connectivity for institutional on-chain trading</t>
+          <t>Fund-administration back-office software (fund accounting, LP reporting, fundraising workflows) for 500+ GPs and fund administrators supporting $185B+ in assets</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -770,17 +770,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-26</t>
+          <t>15-Jul-26</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>c. myers corporation</t>
+          <t>bloXroute Labs</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Strata Decision Technology (Roper)</t>
+          <t>FalconX</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
+          <t>Blockchain distribution network delivering low-latency transaction propagation, real-time chain data, and trading connectivity for institutional on-chain trading</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>16-Jul-26</t>
+          <t>14-Jul-26</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Veridas</t>
+          <t>c. myers corporation</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Fourthline</t>
+          <t>Strata Decision Technology (Roper)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
+          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -931,93 +931,271 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>16-Jul-26</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Veridas</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Fourthline</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>17-Jul-26</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Strategic M&amp;A</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>14-Jul-26</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Qolo</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>CSI (Computer Services, Inc.)</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>API-based treasury and payments infrastructure unifying card issuing, multi-rail money movement, and real-time ledgering for commercial banks and embedded finance</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>17-Jul-26</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>14-Jul-26</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Cherre</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>RealPage (Thoma Bravo)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Real estate data-intelligence platform resolving 4B+ property entities (~$4T in assets) into standardized, governed datasets for institutional owners, investment managers, and operators</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R6"/>
+  <autoFilter ref="A1:R8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lock two new conventions (USA/UK country abbreviations; sector A-Z then newest-first sort); reclassify Velocity to Corporate Financial Function
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBdTT3suK4uAL7A2zUGPUX
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-17.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-26</t>
+          <t>16-Jul-26</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>c. myers corporation</t>
+          <t>Veridas</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Strata Decision Technology (Roper)</t>
+          <t>Fourthline</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
+          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -946,17 +946,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>16-Jul-26</t>
+          <t>14-Jul-26</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Veridas</t>
+          <t>c. myers corporation</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Fourthline</t>
+          <t>Strata Decision Technology (Roper)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Biometric identity-verification and anti-fraud platform; all-stock merger with Fourthline's KYC/AML orchestration business creating a transatlantic identity-compliance platform (BBVA and other holders roll over)</t>
+          <t>ALM, budgeting, and strategic-planning advisory and decision support for 600+ banks and credit unions; being combined with Strata's Axiom FP&amp;A software</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1306,29 +1306,29 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-26</t>
+          <t>15-Jul-26</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Flex</t>
+          <t>Lumin Digital</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Halo Fund</t>
+          <t>Light Street Capital; 15 existing FI clients via SPV</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>AI-native business- and private-banking platform for business owners (banking, cards, bill pay, treasury); launching stablecoin-powered cross-border payments</t>
+          <t>Cloud-native digital banking platform (online/mobile banking, account opening, engagement) for US banks and credit unions; $70M+ of the round from 15 existing FI clients</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -1365,29 +1365,29 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>15-Jul-26</t>
+          <t>14-Jul-26</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Lumin Digital</t>
+          <t>Flex</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Light Street Capital; 15 existing FI clients via SPV</t>
+          <t>Halo Fund</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Cloud-native digital banking platform (online/mobile banking, account opening, engagement) for US banks and credit unions; $70M+ of the round from 15 existing FI clients</t>
+          <t>AI-native business- and private-banking platform for business owners (banking, cards, bill pay, treasury); launching stablecoin-powered cross-border payments</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1554,16 +1554,16 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Hadrius</t>
+          <t>Velocity</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>CRV</t>
+          <t>Dragonfly, FirstMark</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Agentic AI compliance platform (marketing review, comms surveillance, trade monitoring) for 500+ RIAs, broker-dealers, and financial institutions; combined seed + Series A</t>
+          <t>Enterprise stablecoin treasury and settlement infrastructure eliminating prefunding and speeding cross-border liquidity for merchants, PSPs, and financial institutions</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1615,19 +1615,21 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Cover Genius</t>
+          <t>Hadrius</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Vista Credit Partners</t>
+          <t>CRV</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1900</v>
+        <v>27</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -1641,7 +1643,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>B2B2C embedded-insurance platform (XCover) letting digital platforms sell protection at checkout across 200+ distribution partners; structured growth capital from Vista's credit arm</t>
+          <t>Agentic AI compliance platform (marketing review, comms surveillance, trade monitoring) for 500+ RIAs, broker-dealers, and financial institutions; combined seed + Series A</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1664,26 +1666,26 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-26</t>
+          <t>15-Jul-26</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Feathery</t>
+          <t>American Growth Insurance</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Portage Ventures</t>
+          <t>Rockbridge Growth Equity, Atomic</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1702,7 +1704,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>AI operating and decisioning system automating intake, underwriting, and servicing workflows for 300+ insurance and wealth-management firms</t>
+          <t>AI-enabled specialty insurance brokerage roll-up acquiring independent US agencies and rebuilding them on a proprietary AI-native stack; ~$70M committed equity at launch</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1725,31 +1727,29 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>15-Jul-26</t>
+          <t>14-Jul-26</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>American Growth Insurance</t>
+          <t>Cover Genius</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Rockbridge Growth Equity, Atomic</t>
+          <t>Vista Credit Partners</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>1900</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>AI-enabled specialty insurance brokerage roll-up acquiring independent US agencies and rebuilding them on a proprietary AI-native stack; ~$70M committed equity at launch</t>
+          <t>B2B2C embedded-insurance platform (XCover) letting digital platforms sell protection at checkout across 200+ distribution partners; structured growth capital from Vista's credit arm</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1796,16 +1796,16 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Velocity</t>
+          <t>Feathery</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Dragonfly, FirstMark</t>
+          <t>Portage Ventures</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Enterprise stablecoin treasury and settlement infrastructure eliminating prefunding and speeding cross-border liquidity for merchants, PSPs, and financial institutions</t>
+          <t>AI operating and decisioning system automating intake, underwriting, and servicing workflows for 300+ insurance and wealth-management firms</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">

</xml_diff>